<commit_message>
Reality reset: 44 modules all roadmap; iTrak gap analysis logged
- All Excel rows status reset to 'roadmap'; previous live/soon labels were aspirational, not build state
- Added 4 modules from iTrak gap analysis: Contacts (Admin / Core), Vehicles (Surveillance), Lost & Found (Operations), Visitor Management (Guests)
- Renamed Warnings to Disciplinary Actions
- Split Onboarding + Job Board into two modules
- CLAUDE.md count updated 39 -> 44
- decisions.md gains two entries: reality reset + iTrak gap analysis (4 added, 12 permanently skipped)
- specs/CRS_Blueprint.html regen deferred (scripts/v21_content.py still has stale 'Shift Log' / 'Daily Brief' names)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CRS_Module_OptionSets.xlsx
+++ b/data/CRS_Module_OptionSets.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -836,9 +836,9 @@
           <t>Admin / Core</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -884,9 +884,9 @@
           <t>Admin / Core</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G3" s="3" t="n">
@@ -932,9 +932,9 @@
           <t>Admin / Core</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -980,9 +980,9 @@
           <t>Admin / Core</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -1028,9 +1028,9 @@
           <t>Admin / Core</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G6" s="3" t="n">
@@ -1076,9 +1076,9 @@
           <t>Admin / Core</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
@@ -1124,9 +1124,9 @@
           <t>Admin / Core</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G8" s="3" t="n">
@@ -1198,35 +1198,35 @@
     </row>
     <row r="10" ht="60" customHeight="1">
       <c r="A10" s="3" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>reporting</t>
+          <t>contacts</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Reporting</t>
+          <t>Contacts</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>file-earmark-text</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+          <t>person-rolodex</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Admin / Core</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G10" s="3" t="n">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
@@ -1235,32 +1235,32 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>reports</t>
+          <t>contacts</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>Document every incident, error, and procedure violation across the property. Attach evidence, assign to the responsible department, track responses, and close with a formal resolution.</t>
+          <t>Database of professional contacts — vendors, agencies, regulators, suppliers. Linked to Reports, Investigations, and Incidents.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>task_management</t>
+          <t>reporting</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Task Manager</t>
+          <t>Reporting</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>check2-square</t>
+          <t>file-earmark-text</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1268,13 +1268,13 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G11" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
@@ -1283,32 +1283,32 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>tasks</t>
+          <t>reports</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Assign work to individuals or teams, track progress through statuses, break tasks into subtasks, and collaborate via comments. Every department manages its own tasks, with visibility controlled by the department head.</t>
+          <t>Document every incident, error, and procedure violation across the property. Attach evidence, assign to the responsible department, track responses, and close with a formal resolution.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>rfi</t>
+          <t>task_management</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Request for Investigation</t>
+          <t>Task Manager</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>search</t>
+          <t>check2-square</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -1316,13 +1316,13 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G12" s="3" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
@@ -1331,32 +1331,32 @@
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>rfi</t>
+          <t>tasks</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Formally request investigations from another department — share context, attach evidence, and track acceptance. The receiving department assigns the work and reports back when complete.</t>
+          <t>Assign work to individuals or teams, track progress through statuses, break tasks into subtasks, and collaborate via comments. Every department manages its own tasks, with visibility controlled by the department head.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>dashboard</t>
+          <t>rfi</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Dashboard</t>
+          <t>Request for Investigation</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>speedometer2</t>
+          <t>search</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -1364,13 +1364,13 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G13" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
@@ -1379,32 +1379,32 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>dashboard</t>
+          <t>rfi</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Your personal home screen showing what needs your attention right now — open reports, assigned tasks, unread notifications, and key KPIs across the modules you work with.</t>
+          <t>Formally request investigations from another department — share context, attach evidence, and track acceptance. The receiving department assigns the work and reports back when complete.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>malfunction_log</t>
+          <t>dashboard</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Malfunction Log</t>
+          <t>Dashboard</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>exclamation-triangle</t>
+          <t>speedometer2</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -1412,13 +1412,13 @@
           <t>Operations</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G14" s="3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
@@ -1427,46 +1427,46 @@
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>malfunction</t>
+          <t>dashboard</t>
         </is>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Track equipment and facility malfunctions across every department — cameras, access control, gaming equipment, cage systems, F&amp;B. Route to maintenance, track resolution time, and spot recurring faults.</t>
+          <t>Your personal home screen showing what needs your attention right now — open reports, assigned tasks, unread notifications, and key KPIs across the modules you work with.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
       <c r="A15" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>daily_activity_log</t>
+          <t>malfunction_log</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Daily Activity Log</t>
+          <t>Malfunction Log</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>clipboard2-pulse</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Surveillance</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+          <t>exclamation-triangle</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G15" s="3" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
@@ -1475,46 +1475,46 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>dal</t>
+          <t>malfunction</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Operator's running log maintained in real time during the shift. Record every observation, event, and minor incident as it happens. Reviewed by the shift supervisor at end of shift.</t>
+          <t>Track equipment and facility malfunctions across every department — cameras, access control, gaming equipment, cage systems, F&amp;B. Route to maintenance, track resolution time, and spot recurring faults.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="3" t="n">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>end_of_shift_report</t>
+          <t>lost_found</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>End of Shift Report</t>
+          <t>Lost &amp; Found</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>journal-bookmark</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Surveillance</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+          <t>box-seam</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G16" s="3" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
@@ -1523,32 +1523,32 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>eos</t>
+          <t>lost-and-found</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Supervisor's consolidated report at the end of the gaming date. Covers financials (drop/win/hold), pax count, major winners and losers, cage issues, reports generated, key events, and operator assignments. Sent to surveillance management and department heads.</t>
+          <t>Lost and found item lifecycle — intake, storage, claim, return, disposal.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="3" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>investigation_cases</t>
+          <t>daily_activity_log</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Investigation Cases</t>
+          <t>Daily Activity Log</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>folder2-open</t>
+          <t>clipboard2-pulse</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
@@ -1571,32 +1571,32 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>investigations</t>
+          <t>dal</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Turn repeat incidents and suspicious patterns into structured investigation cases. Link related reports, track leads, document findings, and close with a formal outcome.</t>
+          <t>Operator's running log maintained in real time during the shift. Record every observation, event, and minor incident as it happens. Reviewed by the shift supervisor at end of shift.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="3" t="n">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>alert_center</t>
+          <t>end_of_shift_report</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Alert Center</t>
+          <t>End of Shift Report</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>broadcast</t>
+          <t>journal-bookmark</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
@@ -1619,32 +1619,32 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>alerts</t>
+          <t>eos</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Real-time alert system across the property. Floor staff trigger alerts via tablets at gaming tables — F100 operator alerts (buy-ins, disputes, supervisor needed) and F1000 distress alarms. Surveillance receives instant push notifications. Track every alert by location, time, type, response time, and resolution with full audit trail and analytics dashboard.</t>
+          <t>Supervisor's consolidated report at the end of the gaming date. Covers financials (drop/win/hold), pax count, major winners and losers, cage issues, reports generated, key events, and operator assignments. Sent to surveillance management and department heads.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="3" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>cctv_audits</t>
+          <t>investigation_cases</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>CCTV Audits</t>
+          <t>Investigation Cases</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>camera-video</t>
+          <t>folder2-open</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1652,13 +1652,13 @@
           <t>Surveillance</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G19" s="3" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
@@ -1667,32 +1667,32 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>cctv-audits</t>
+          <t>investigations</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Structured audits performed by reviewing recorded footage against predefined templates — Dealer Performance, Player Rating, Pit Rotation, Cashier Transaction, and more. Each template has its own checklist; completed audits track findings and link to follow-up reports.</t>
+          <t>Turn repeat incidents and suspicious patterns into structured investigation cases. Link related reports, track leads, document findings, and close with a formal outcome.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="3" t="n">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>equipment_inspection</t>
+          <t>alert_center</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Equipment Inspection Log</t>
+          <t>Alert Center</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>tools</t>
+          <t>broadcast</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1700,13 +1700,13 @@
           <t>Surveillance</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G20" s="3" t="n">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
@@ -1715,46 +1715,46 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>equipment-inspection</t>
+          <t>alerts</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>Scheduled inspections of surveillance equipment — DVR/NVR health, backup systems, recording retention, redundancy checks. Track completion, findings, and follow-up actions.</t>
+          <t>Real-time alert system across the property. Floor staff trigger alerts via tablets at gaming tables — F100 operator alerts (buy-ins, disputes, supervisor needed) and F1000 distress alarms. Surveillance receives instant push notifications. Track every alert by location, time, type, response time, and resolution with full audit trail and analytics dashboard.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="3" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>guest_management</t>
+          <t>cctv_audits</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Guest Management</t>
+          <t>CCTV Audits</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>person-circle</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>Guests</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+          <t>camera-video</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>Surveillance</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
@@ -1763,37 +1763,37 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>guests</t>
+          <t>cctv-audits</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>Central directory for every guest visiting your property — identification, visit history, photos, linked reports, VIP status, and internal notes from your team.</t>
+          <t>Structured audits performed by reviewing recorded footage against predefined templates — Dealer Performance, Player Rating, Pit Rotation, Cashier Transaction, and more. Each template has its own checklist; completed audits track findings and link to follow-up reports.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>guest_barring</t>
+          <t>equipment_inspection</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Guest Barring</t>
+          <t>Equipment Inspection Log</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>slash-circle</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>Guests</t>
+          <t>tools</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Surveillance</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -1802,7 +1802,7 @@
         </is>
       </c>
       <c r="G22" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
@@ -1811,37 +1811,37 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>guest-barring</t>
+          <t>equipment-inspection</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Formal process to bar guests from the property — capture the reason, duration, evidence, and jurisdiction scope. Alerts your team if a barred guest attempts to re-enter.</t>
+          <t>Scheduled inspections of surveillance equipment — DVR/NVR health, backup systems, recording retention, redundancy checks. Track completion, findings, and follow-up actions.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="3" t="n">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>guest_watchlist</t>
+          <t>vehicles</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Guest Watchlist</t>
+          <t>Vehicles</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>bookmark-star</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Guests</t>
+          <t>car-front</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>Surveillance</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1850,7 +1850,7 @@
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
@@ -1859,32 +1859,32 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>guest-watchlist</t>
+          <t>vehicles</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>Manage self-exclusions, cooling-off agreements, and internal watchlists in one place. Compliance-tracked with legal-hold and automated regulator reporting.</t>
+          <t>Vehicle records — license plate, make, model, owner, associated subjects and incidents.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>guest_statistics</t>
+          <t>guest_management</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Guest Statistics</t>
+          <t>Guest Management</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>bar-chart</t>
+          <t>person-circle</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="G24" s="3" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
@@ -1907,32 +1907,32 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>guest-stats</t>
+          <t>guests</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Understand your guest base — visit frequency patterns, spend bands, incident rates by segment, and trend detection. Data to support responsible-gambling and marketing decisions.</t>
+          <t>Central directory for every guest visiting your property — identification, visit history, photos, linked reports, VIP status, and internal notes from your team.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="3" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>vip_loyalty</t>
+          <t>guest_barring</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>VIP / Loyalty Tracking</t>
+          <t>Guest Barring</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>star</t>
+          <t>slash-circle</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="G25" s="3" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
@@ -1955,46 +1955,46 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>vip</t>
+          <t>guest-barring</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>Manage VIP guests and loyalty programs — assigned hosts, preferences, comp tracking, and high-value guest alerts. Integrates with your external loyalty platform if you have one.</t>
+          <t>Formal process to bar guests from the property — capture the reason, duration, evidence, and jurisdiction scope. Alerts your team if a barred guest attempts to re-enter.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>employee_management</t>
+          <t>guest_watchlist</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Employee Management</t>
+          <t>Guest Watchlist</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>people</t>
-        </is>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>HR / Employees</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+          <t>bookmark-star</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Guests</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G26" s="3" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
@@ -2003,46 +2003,46 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>guest-watchlist</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>Central employee directory — profiles, departments, positions, documents, notes, and complete history. Organisation-wide search, multi-property support, and GDPR-compliant anonymization on termination.</t>
+          <t>Manage self-exclusions, cooling-off agreements, and internal watchlists in one place. Compliance-tracked with legal-hold and automated regulator reporting.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" s="3" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>onboarding_jobboard</t>
+          <t>guest_statistics</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Onboarding + Job Board</t>
+          <t>Guest Statistics</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>briefcase</t>
-        </is>
-      </c>
-      <c r="E27" s="10" t="inlineStr">
-        <is>
-          <t>HR / Employees</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>live</t>
+          <t>bar-chart</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Guests</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G27" s="3" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
@@ -2051,37 +2051,37 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>onboarding</t>
+          <t>guest-stats</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>Public careers page for your property — publish openings, collect applications, and onboard new hires through a guided workflow. Integrates with Employee Management on hire.</t>
+          <t>Understand your guest base — visit frequency patterns, spend bands, incident rates by segment, and trend detection. Data to support responsible-gambling and marketing decisions.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>warnings</t>
+          <t>vip_loyalty</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Warnings</t>
+          <t>VIP / Loyalty Tracking</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>exclamation-octagon</t>
-        </is>
-      </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>HR / Employees</t>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Guests</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="G28" s="3" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
@@ -2099,37 +2099,37 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>warnings</t>
+          <t>vip</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>Manage formal employee warnings — verbal, written, and final. Link evidence from reports, set escalation rules, and maintain a complete disciplinary trail for every employee.</t>
+          <t>Manage VIP guests and loyalty programs — assigned hosts, preferences, comp tracking, and high-value guest alerts. Integrates with your external loyalty platform if you have one.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="3" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>appraisals</t>
+          <t>visitor_management</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Appraisals</t>
+          <t>Visitor Management</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>hand-thumbs-up</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>HR / Employees</t>
+          <t>person-badge</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Guests</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="G29" s="3" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
@@ -2147,32 +2147,32 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>appraisals</t>
+          <t>visitor-management</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>Run employee performance reviews on a schedule you define — set KPIs, collect feedback from multiple raters, agree on growth plans, and track progress between cycles.</t>
+          <t>Pre-register and check in/out non-guest visitors — contractors, vendors, deliveries, VIP visitors. Distinct from Guest Management.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="3" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>attendance</t>
+          <t>employee_management</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Attendance</t>
+          <t>Employee Management</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>clock-history</t>
+          <t>people</t>
         </is>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -2186,7 +2186,7 @@
         </is>
       </c>
       <c r="G30" s="3" t="n">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
@@ -2195,32 +2195,32 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>attendance</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Track when employees clock in and out, flag late arrivals and absences, and summarise attendance by employee or department. Feeds into Scheduling and Payroll.</t>
+          <t>Central employee directory — profiles, departments, positions, documents, notes, and complete history. Organisation-wide search, multi-property support, and GDPR-compliant anonymization on termination.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" s="3" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>scheduling</t>
+          <t>onboarding</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>calendar-week</t>
+          <t>person-plus</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="G31" s="3" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
@@ -2243,32 +2243,32 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>scheduling</t>
+          <t>onboarding</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Replace your scheduling spreadsheets. Build rosters with any pattern your departments use — 5/2, 4/2, rotating 2/2 day/night. Handle shift swaps and day-off requests with routing to department heads.</t>
+          <t>Guided onboarding flow for new hires — collect documents, assign training, and integrate with Employee Management on hire.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="3" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>leave_management</t>
+          <t>job_board</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Leave Management</t>
+          <t>Job Board</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>airplane</t>
+          <t>briefcase</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -2282,7 +2282,7 @@
         </is>
       </c>
       <c r="G32" s="3" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
@@ -2291,32 +2291,32 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>leave</t>
+          <t>job-board</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Track PTO, sick leave, and unpaid leave for every employee. Maintain balances, route requests for approval, and show who's out on a shared calendar.</t>
+          <t>Public careers page for your property — publish openings and collect applications. Hand-off to Onboarding on hire.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" s="3" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>payroll</t>
+          <t>disciplinary_actions</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Disciplinary Actions</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>cash-stack</t>
+          <t>exclamation-octagon</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="G33" s="3" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
@@ -2339,37 +2339,37 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>payroll</t>
+          <t>disciplinary-actions</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>Run payroll based on scheduled hours, attendance, and overtime. Apply deductions, generate payslips, and export to your accounting system.</t>
+          <t>Manage formal employee disciplinary actions — verbal, written, and final. Link evidence from reports, set escalation rules, and maintain a complete disciplinary trail for every employee.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="3" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>compliance_register</t>
+          <t>appraisals</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Compliance Register</t>
+          <t>Appraisals</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>shield-check</t>
-        </is>
-      </c>
-      <c r="E34" s="11" t="inlineStr">
-        <is>
-          <t>Compliance</t>
+          <t>hand-thumbs-up</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>HR / Employees</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2378,7 +2378,7 @@
         </is>
       </c>
       <c r="G34" s="3" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
@@ -2387,37 +2387,37 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>compliance</t>
+          <t>appraisals</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>Central register of every regulatory obligation your property must meet — the controls in place, supporting evidence, responsible owners, and review cadence. Audit-ready at any time.</t>
+          <t>Run employee performance reviews on a schedule you define — set KPIs, collect feedback from multiple raters, agree on growth plans, and track progress between cycles.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
       <c r="A35" s="3" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>regulatory_reports</t>
+          <t>attendance</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Regulatory Reports</t>
+          <t>Attendance</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>file-earmark-ruled</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="inlineStr">
-        <is>
-          <t>Compliance</t>
+          <t>clock-history</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>HR / Employees</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
@@ -2435,37 +2435,37 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>regulatory</t>
+          <t>attendance</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>Generate the periodic reports your regulators require — incident summaries, large transaction reports, compliance attestations. Scheduled, reviewed, and filed with an audit trail.</t>
+          <t>Track when employees clock in and out, flag late arrivals and absences, and summarise attendance by employee or department. Feeds into Scheduling and Payroll.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
       <c r="A36" s="3" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>policy_library</t>
+          <t>scheduling</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Policy Library</t>
+          <t>Scheduling</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>book</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="inlineStr">
-        <is>
-          <t>Compliance</t>
+          <t>calendar-week</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>HR / Employees</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
@@ -2483,37 +2483,37 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>policies</t>
+          <t>scheduling</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>Publish your internal policies and SOPs with version control. Track who has acknowledged which version, and schedule automatic re-reviews so policies stay current.</t>
+          <t>Replace your scheduling spreadsheets. Build rosters with any pattern your departments use — 5/2, 4/2, rotating 2/2 day/night. Handle shift swaps and day-off requests with routing to department heads.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="3" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>leave_management</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Inventory / Sensitive Equipment</t>
+          <t>Leave Management</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>box-seam</t>
-        </is>
-      </c>
-      <c r="E37" s="11" t="inlineStr">
-        <is>
-          <t>Compliance</t>
+          <t>airplane</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>HR / Employees</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -2522,7 +2522,7 @@
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
@@ -2531,46 +2531,46 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>leave</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>Track sensitive gaming equipment — dice, cards, chip sets, cameras. Record serial numbers, maintain custody chain, and perform tamper-evidence checks to satisfy compliance requirements.</t>
+          <t>Track PTO, sick leave, and unpaid leave for every employee. Maintain balances, route requests for approval, and show who's out on a shared calendar.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="3" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>info_board</t>
+          <t>payroll</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Info Board</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>pin-angle</t>
-        </is>
-      </c>
-      <c r="E38" s="12" t="inlineStr">
-        <is>
-          <t>Communication</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>soon</t>
+          <t>cash-stack</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>HR / Employees</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
@@ -2579,37 +2579,37 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>info-board</t>
+          <t>payroll</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>Department-wide noticeboard for shift briefings, new procedures, and team announcements. Target posts to specific roles or departments. Replaces whiteboards and WhatsApp groups.</t>
+          <t>Run payroll based on scheduled hours, attendance, and overtime. Apply deductions, generate payslips, and export to your accounting system.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>announcements</t>
+          <t>compliance_register</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Announcements</t>
+          <t>Compliance Register</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>megaphone</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="inlineStr">
-        <is>
-          <t>Communication</t>
+          <t>shield-check</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Compliance</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2618,7 +2618,7 @@
         </is>
       </c>
       <c r="G39" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
@@ -2627,58 +2627,298 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>announcements</t>
+          <t>compliance</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>Property-wide or targeted announcements — all-hands updates, shift notices, emergency alerts. Track who has read each announcement to confirm message delivery.</t>
+          <t>Central register of every regulatory obligation your property must meet — the controls in place, supporting evidence, responsible owners, and review cadence. Audit-ready at any time.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
       <c r="A40" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>regulatory_reports</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Regulatory Reports</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>file-earmark-ruled</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>regulatory</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Generate the periodic reports your regulators require — incident summaries, large transaction reports, compliance attestations. Scheduled, reviewed, and filed with an audit trail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>policy_library</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Policy Library</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>policies</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Publish your internal policies and SOPs with version control. Track who has acknowledged which version, and schedule automatic re-reviews so policies stay current.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="60" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Inventory / Sensitive Equipment</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>box-seam</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Compliance</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>inventory</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Track sensitive gaming equipment — dice, cards, chip sets, cameras. Record serial numbers, maintain custody chain, and perform tamper-evidence checks to satisfy compliance requirements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="60" customHeight="1">
+      <c r="A43" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>info_board</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Info Board</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>pin-angle</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>info-board</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Department-wide noticeboard for shift briefings, new procedures, and team announcements. Target posts to specific roles or departments. Replaces whiteboards and WhatsApp groups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="60" customHeight="1">
+      <c r="A44" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Announcements</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>megaphone</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Property-wide or targeted announcements — all-hands updates, shift notices, emergency alerts. Track who has read each announcement to confirm message delivery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="60" customHeight="1">
+      <c r="A45" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>internal_messaging</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Internal Messaging</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>chat-dots</t>
         </is>
       </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="E45" s="12" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>roadmap</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="n">
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I40" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
         <is>
           <t>messaging</t>
         </is>
       </c>
-      <c r="J40" s="3" t="inlineStr">
+      <c r="J45" s="3" t="inlineStr">
         <is>
           <t>Work chat scoped to your property. Department channels, direct messages, and file sharing — keeping work communication off WhatsApp and in a compliant, searchable system.</t>
         </is>

</xml_diff>

<commit_message>
Add Break List module 45 — pilot-requested floor allocation
- Added Break List (Operations, sort 70, route break-list, icon arrow-left-right) — pilot explicitly requested
- Real-time pit boss workflow distinct from Scheduling (real-time vs weekly, Pit Boss vs HR ownership)
- xlsx: 45 modules total, all roadmap
- CLAUDE.md: count 44 -> 45
- decisions.md: new top entry with scope distinction vs Scheduling and open build-phase questions

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/CRS_Module_OptionSets.xlsx
+++ b/data/CRS_Module_OptionSets.xlsx
@@ -745,7 +745,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1534,26 +1534,26 @@
     </row>
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="3" t="n">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>daily_activity_log</t>
+          <t>break_list</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Daily Activity Log</t>
+          <t>Break List</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>clipboard2-pulse</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>Surveillance</t>
+          <t>arrow-left-right</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Operations</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="G17" s="3" t="n">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
@@ -1571,32 +1571,32 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>dal</t>
+          <t>break-list</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Operator's running log maintained in real time during the shift. Record every observation, event, and minor incident as it happens. Reviewed by the shift supervisor at end of shift.</t>
+          <t>Real-time floor allocation. Pit boss assigns on-shift dealers and inspectors to gaming tables in 20–30 minute rotations and tracks breaks. Distinct from Scheduling — Scheduling plans the week, Break List runs the shift.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>end_of_shift_report</t>
+          <t>daily_activity_log</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>End of Shift Report</t>
+          <t>Daily Activity Log</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>journal-bookmark</t>
+          <t>clipboard2-pulse</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="G18" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
@@ -1619,32 +1619,32 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>eos</t>
+          <t>dal</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>Supervisor's consolidated report at the end of the gaming date. Covers financials (drop/win/hold), pax count, major winners and losers, cage issues, reports generated, key events, and operator assignments. Sent to surveillance management and department heads.</t>
+          <t>Operator's running log maintained in real time during the shift. Record every observation, event, and minor incident as it happens. Reviewed by the shift supervisor at end of shift.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="3" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>investigation_cases</t>
+          <t>end_of_shift_report</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Investigation Cases</t>
+          <t>End of Shift Report</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>folder2-open</t>
+          <t>journal-bookmark</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="G19" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
@@ -1667,32 +1667,32 @@
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>investigations</t>
+          <t>eos</t>
         </is>
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Turn repeat incidents and suspicious patterns into structured investigation cases. Link related reports, track leads, document findings, and close with a formal outcome.</t>
+          <t>Supervisor's consolidated report at the end of the gaming date. Covers financials (drop/win/hold), pax count, major winners and losers, cage issues, reports generated, key events, and operator assignments. Sent to surveillance management and department heads.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="3" t="n">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>alert_center</t>
+          <t>investigation_cases</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Alert Center</t>
+          <t>Investigation Cases</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>broadcast</t>
+          <t>folder2-open</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1706,7 +1706,7 @@
         </is>
       </c>
       <c r="G20" s="3" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
@@ -1715,32 +1715,32 @@
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>alerts</t>
+          <t>investigations</t>
         </is>
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>Real-time alert system across the property. Floor staff trigger alerts via tablets at gaming tables — F100 operator alerts (buy-ins, disputes, supervisor needed) and F1000 distress alarms. Surveillance receives instant push notifications. Track every alert by location, time, type, response time, and resolution with full audit trail and analytics dashboard.</t>
+          <t>Turn repeat incidents and suspicious patterns into structured investigation cases. Link related reports, track leads, document findings, and close with a formal outcome.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="3" t="n">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>cctv_audits</t>
+          <t>alert_center</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>CCTV Audits</t>
+          <t>Alert Center</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>camera-video</t>
+          <t>broadcast</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -1754,7 +1754,7 @@
         </is>
       </c>
       <c r="G21" s="3" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
@@ -1763,32 +1763,32 @@
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>cctv-audits</t>
+          <t>alerts</t>
         </is>
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>Structured audits performed by reviewing recorded footage against predefined templates — Dealer Performance, Player Rating, Pit Rotation, Cashier Transaction, and more. Each template has its own checklist; completed audits track findings and link to follow-up reports.</t>
+          <t>Real-time alert system across the property. Floor staff trigger alerts via tablets at gaming tables — F100 operator alerts (buy-ins, disputes, supervisor needed) and F1000 distress alarms. Surveillance receives instant push notifications. Track every alert by location, time, type, response time, and resolution with full audit trail and analytics dashboard.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>equipment_inspection</t>
+          <t>cctv_audits</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Equipment Inspection Log</t>
+          <t>CCTV Audits</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>tools</t>
+          <t>camera-video</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -1802,7 +1802,7 @@
         </is>
       </c>
       <c r="G22" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
@@ -1811,32 +1811,32 @@
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>equipment-inspection</t>
+          <t>cctv-audits</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Scheduled inspections of surveillance equipment — DVR/NVR health, backup systems, recording retention, redundancy checks. Track completion, findings, and follow-up actions.</t>
+          <t>Structured audits performed by reviewing recorded footage against predefined templates — Dealer Performance, Player Rating, Pit Rotation, Cashier Transaction, and more. Each template has its own checklist; completed audits track findings and link to follow-up reports.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
       <c r="A23" s="3" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>vehicles</t>
+          <t>equipment_inspection</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Vehicles</t>
+          <t>Equipment Inspection Log</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>car-front</t>
+          <t>tools</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1850,7 +1850,7 @@
         </is>
       </c>
       <c r="G23" s="3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
@@ -1859,37 +1859,37 @@
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>vehicles</t>
+          <t>equipment-inspection</t>
         </is>
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>Vehicle records — license plate, make, model, owner, associated subjects and incidents.</t>
+          <t>Scheduled inspections of surveillance equipment — DVR/NVR health, backup systems, recording retention, redundancy checks. Track completion, findings, and follow-up actions.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
       <c r="A24" s="3" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>guest_management</t>
+          <t>vehicles</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Guest Management</t>
+          <t>Vehicles</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>person-circle</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
-        <is>
-          <t>Guests</t>
+          <t>car-front</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Surveillance</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1898,7 +1898,7 @@
         </is>
       </c>
       <c r="G24" s="3" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
@@ -1907,32 +1907,32 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>guests</t>
+          <t>vehicles</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Central directory for every guest visiting your property — identification, visit history, photos, linked reports, VIP status, and internal notes from your team.</t>
+          <t>Vehicle records — license plate, make, model, owner, associated subjects and incidents.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
       <c r="A25" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>guest_barring</t>
+          <t>guest_management</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Guest Barring</t>
+          <t>Guest Management</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>slash-circle</t>
+          <t>person-circle</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="G25" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
@@ -1955,32 +1955,32 @@
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>guest-barring</t>
+          <t>guests</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>Formal process to bar guests from the property — capture the reason, duration, evidence, and jurisdiction scope. Alerts your team if a barred guest attempts to re-enter.</t>
+          <t>Central directory for every guest visiting your property — identification, visit history, photos, linked reports, VIP status, and internal notes from your team.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
       <c r="A26" s="3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>guest_watchlist</t>
+          <t>guest_barring</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Guest Watchlist</t>
+          <t>Guest Barring</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>bookmark-star</t>
+          <t>slash-circle</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -1994,7 +1994,7 @@
         </is>
       </c>
       <c r="G26" s="3" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
@@ -2003,32 +2003,32 @@
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>guest-watchlist</t>
+          <t>guest-barring</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>Manage self-exclusions, cooling-off agreements, and internal watchlists in one place. Compliance-tracked with legal-hold and automated regulator reporting.</t>
+          <t>Formal process to bar guests from the property — capture the reason, duration, evidence, and jurisdiction scope. Alerts your team if a barred guest attempts to re-enter.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
       <c r="A27" s="3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>guest_statistics</t>
+          <t>guest_watchlist</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Guest Statistics</t>
+          <t>Guest Watchlist</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>bar-chart</t>
+          <t>bookmark-star</t>
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr">
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="G27" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
@@ -2051,32 +2051,32 @@
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>guest-stats</t>
+          <t>guest-watchlist</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>Understand your guest base — visit frequency patterns, spend bands, incident rates by segment, and trend detection. Data to support responsible-gambling and marketing decisions.</t>
+          <t>Manage self-exclusions, cooling-off agreements, and internal watchlists in one place. Compliance-tracked with legal-hold and automated regulator reporting.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>vip_loyalty</t>
+          <t>guest_statistics</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>VIP / Loyalty Tracking</t>
+          <t>Guest Statistics</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>star</t>
+          <t>bar-chart</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="G28" s="3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
@@ -2099,32 +2099,32 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>vip</t>
+          <t>guest-stats</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>Manage VIP guests and loyalty programs — assigned hosts, preferences, comp tracking, and high-value guest alerts. Integrates with your external loyalty platform if you have one.</t>
+          <t>Understand your guest base — visit frequency patterns, spend bands, incident rates by segment, and trend detection. Data to support responsible-gambling and marketing decisions.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
       <c r="A29" s="3" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>visitor_management</t>
+          <t>vip_loyalty</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Visitor Management</t>
+          <t>VIP / Loyalty Tracking</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>person-badge</t>
+          <t>star</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="G29" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
@@ -2147,37 +2147,37 @@
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>visitor-management</t>
+          <t>vip</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>Pre-register and check in/out non-guest visitors — contractors, vendors, deliveries, VIP visitors. Distinct from Guest Management.</t>
+          <t>Manage VIP guests and loyalty programs — assigned hosts, preferences, comp tracking, and high-value guest alerts. Integrates with your external loyalty platform if you have one.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
       <c r="A30" s="3" t="n">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>employee_management</t>
+          <t>visitor_management</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Employee Management</t>
+          <t>Visitor Management</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>people</t>
-        </is>
-      </c>
-      <c r="E30" s="10" t="inlineStr">
-        <is>
-          <t>HR / Employees</t>
+          <t>person-badge</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Guests</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -2186,7 +2186,7 @@
         </is>
       </c>
       <c r="G30" s="3" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
@@ -2195,32 +2195,32 @@
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>employees</t>
+          <t>visitor-management</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Central employee directory — profiles, departments, positions, documents, notes, and complete history. Organisation-wide search, multi-property support, and GDPR-compliant anonymization on termination.</t>
+          <t>Pre-register and check in/out non-guest visitors — contractors, vendors, deliveries, VIP visitors. Distinct from Guest Management.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
       <c r="A31" s="3" t="n">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>onboarding</t>
+          <t>employee_management</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Onboarding</t>
+          <t>Employee Management</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>person-plus</t>
+          <t>people</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -2234,7 +2234,7 @@
         </is>
       </c>
       <c r="G31" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
@@ -2243,32 +2243,32 @@
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>onboarding</t>
+          <t>employees</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Guided onboarding flow for new hires — collect documents, assign training, and integrate with Employee Management on hire.</t>
+          <t>Central employee directory — profiles, departments, positions, documents, notes, and complete history. Organisation-wide search, multi-property support, and GDPR-compliant anonymization on termination.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
       <c r="A32" s="3" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>job_board</t>
+          <t>onboarding</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Job Board</t>
+          <t>Onboarding</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>briefcase</t>
+          <t>person-plus</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -2282,7 +2282,7 @@
         </is>
       </c>
       <c r="G32" s="3" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H32" s="3" t="inlineStr">
         <is>
@@ -2291,32 +2291,32 @@
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>job-board</t>
+          <t>onboarding</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Public careers page for your property — publish openings and collect applications. Hand-off to Onboarding on hire.</t>
+          <t>Guided onboarding flow for new hires — collect documents, assign training, and integrate with Employee Management on hire.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
       <c r="A33" s="3" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>disciplinary_actions</t>
+          <t>job_board</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Disciplinary Actions</t>
+          <t>Job Board</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>exclamation-octagon</t>
+          <t>briefcase</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="G33" s="3" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
@@ -2339,32 +2339,32 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>disciplinary-actions</t>
+          <t>job-board</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>Manage formal employee disciplinary actions — verbal, written, and final. Link evidence from reports, set escalation rules, and maintain a complete disciplinary trail for every employee.</t>
+          <t>Public careers page for your property — publish openings and collect applications. Hand-off to Onboarding on hire.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
       <c r="A34" s="3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>appraisals</t>
+          <t>disciplinary_actions</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Appraisals</t>
+          <t>Disciplinary Actions</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>hand-thumbs-up</t>
+          <t>exclamation-octagon</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
@@ -2378,7 +2378,7 @@
         </is>
       </c>
       <c r="G34" s="3" t="n">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
@@ -2387,32 +2387,32 @@
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>appraisals</t>
+          <t>disciplinary-actions</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>Run employee performance reviews on a schedule you define — set KPIs, collect feedback from multiple raters, agree on growth plans, and track progress between cycles.</t>
+          <t>Manage formal employee disciplinary actions — verbal, written, and final. Link evidence from reports, set escalation rules, and maintain a complete disciplinary trail for every employee.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
       <c r="A35" s="3" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>attendance</t>
+          <t>appraisals</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Attendance</t>
+          <t>Appraisals</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>clock-history</t>
+          <t>hand-thumbs-up</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
@@ -2426,7 +2426,7 @@
         </is>
       </c>
       <c r="G35" s="3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
@@ -2435,32 +2435,32 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>attendance</t>
+          <t>appraisals</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>Track when employees clock in and out, flag late arrivals and absences, and summarise attendance by employee or department. Feeds into Scheduling and Payroll.</t>
+          <t>Run employee performance reviews on a schedule you define — set KPIs, collect feedback from multiple raters, agree on growth plans, and track progress between cycles.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
       <c r="A36" s="3" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>scheduling</t>
+          <t>attendance</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Scheduling</t>
+          <t>Attendance</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>calendar-week</t>
+          <t>clock-history</t>
         </is>
       </c>
       <c r="E36" s="10" t="inlineStr">
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="G36" s="3" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
@@ -2483,32 +2483,32 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>scheduling</t>
+          <t>attendance</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>Replace your scheduling spreadsheets. Build rosters with any pattern your departments use — 5/2, 4/2, rotating 2/2 day/night. Handle shift swaps and day-off requests with routing to department heads.</t>
+          <t>Track when employees clock in and out, flag late arrivals and absences, and summarise attendance by employee or department. Feeds into Scheduling and Payroll.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
       <c r="A37" s="3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>leave_management</t>
+          <t>scheduling</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Leave Management</t>
+          <t>Scheduling</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>airplane</t>
+          <t>calendar-week</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -2522,7 +2522,7 @@
         </is>
       </c>
       <c r="G37" s="3" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
@@ -2531,32 +2531,32 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>leave</t>
+          <t>scheduling</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>Track PTO, sick leave, and unpaid leave for every employee. Maintain balances, route requests for approval, and show who's out on a shared calendar.</t>
+          <t>Replace your scheduling spreadsheets. Build rosters with any pattern your departments use — 5/2, 4/2, rotating 2/2 day/night. Handle shift swaps and day-off requests with routing to department heads.</t>
         </is>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
       <c r="A38" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>payroll</t>
+          <t>leave_management</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Payroll</t>
+          <t>Leave Management</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>cash-stack</t>
+          <t>airplane</t>
         </is>
       </c>
       <c r="E38" s="10" t="inlineStr">
@@ -2570,7 +2570,7 @@
         </is>
       </c>
       <c r="G38" s="3" t="n">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
@@ -2579,37 +2579,37 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>payroll</t>
+          <t>leave</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>Run payroll based on scheduled hours, attendance, and overtime. Apply deductions, generate payslips, and export to your accounting system.</t>
+          <t>Track PTO, sick leave, and unpaid leave for every employee. Maintain balances, route requests for approval, and show who's out on a shared calendar.</t>
         </is>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
       <c r="A39" s="3" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>compliance_register</t>
+          <t>payroll</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Compliance Register</t>
+          <t>Payroll</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>shield-check</t>
-        </is>
-      </c>
-      <c r="E39" s="11" t="inlineStr">
-        <is>
-          <t>Compliance</t>
+          <t>cash-stack</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>HR / Employees</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
@@ -2618,7 +2618,7 @@
         </is>
       </c>
       <c r="G39" s="3" t="n">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
@@ -2627,32 +2627,32 @@
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>compliance</t>
+          <t>payroll</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>Central register of every regulatory obligation your property must meet — the controls in place, supporting evidence, responsible owners, and review cadence. Audit-ready at any time.</t>
+          <t>Run payroll based on scheduled hours, attendance, and overtime. Apply deductions, generate payslips, and export to your accounting system.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
       <c r="A40" s="3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>regulatory_reports</t>
+          <t>compliance_register</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Regulatory Reports</t>
+          <t>Compliance Register</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>file-earmark-ruled</t>
+          <t>shield-check</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="G40" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
@@ -2675,32 +2675,32 @@
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>regulatory</t>
+          <t>compliance</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>Generate the periodic reports your regulators require — incident summaries, large transaction reports, compliance attestations. Scheduled, reviewed, and filed with an audit trail.</t>
+          <t>Central register of every regulatory obligation your property must meet — the controls in place, supporting evidence, responsible owners, and review cadence. Audit-ready at any time.</t>
         </is>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
       <c r="A41" s="3" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>policy_library</t>
+          <t>regulatory_reports</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Policy Library</t>
+          <t>Regulatory Reports</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>book</t>
+          <t>file-earmark-ruled</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
@@ -2714,7 +2714,7 @@
         </is>
       </c>
       <c r="G41" s="3" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
@@ -2723,32 +2723,32 @@
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>policies</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>Publish your internal policies and SOPs with version control. Track who has acknowledged which version, and schedule automatic re-reviews so policies stay current.</t>
+          <t>Generate the periodic reports your regulators require — incident summaries, large transaction reports, compliance attestations. Scheduled, reviewed, and filed with an audit trail.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
       <c r="A42" s="3" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>policy_library</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Inventory / Sensitive Equipment</t>
+          <t>Policy Library</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>box-seam</t>
+          <t>book</t>
         </is>
       </c>
       <c r="E42" s="11" t="inlineStr">
@@ -2762,7 +2762,7 @@
         </is>
       </c>
       <c r="G42" s="3" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="H42" s="3" t="inlineStr">
         <is>
@@ -2771,37 +2771,37 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>policies</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>Track sensitive gaming equipment — dice, cards, chip sets, cameras. Record serial numbers, maintain custody chain, and perform tamper-evidence checks to satisfy compliance requirements.</t>
+          <t>Publish your internal policies and SOPs with version control. Track who has acknowledged which version, and schedule automatic re-reviews so policies stay current.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
       <c r="A43" s="3" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>info_board</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Info Board</t>
+          <t>Inventory / Sensitive Equipment</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>pin-angle</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>Communication</t>
+          <t>box-seam</t>
+        </is>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Compliance</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="G43" s="3" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="H43" s="3" t="inlineStr">
         <is>
@@ -2819,32 +2819,32 @@
       </c>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>info-board</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>Department-wide noticeboard for shift briefings, new procedures, and team announcements. Target posts to specific roles or departments. Replaces whiteboards and WhatsApp groups.</t>
+          <t>Track sensitive gaming equipment — dice, cards, chip sets, cameras. Record serial numbers, maintain custody chain, and perform tamper-evidence checks to satisfy compliance requirements.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
       <c r="A44" s="3" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>announcements</t>
+          <t>info_board</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Announcements</t>
+          <t>Info Board</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>megaphone</t>
+          <t>pin-angle</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -2858,7 +2858,7 @@
         </is>
       </c>
       <c r="G44" s="3" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H44" s="3" t="inlineStr">
         <is>
@@ -2867,58 +2867,106 @@
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>announcements</t>
+          <t>info-board</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>Property-wide or targeted announcements — all-hands updates, shift notices, emergency alerts. Track who has read each announcement to confirm message delivery.</t>
+          <t>Department-wide noticeboard for shift briefings, new procedures, and team announcements. Target posts to specific roles or departments. Replaces whiteboards and WhatsApp groups.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
       <c r="A45" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Announcements</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>megaphone</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>Communication</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>announcements</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Property-wide or targeted announcements — all-hands updates, shift notices, emergency alerts. Track who has read each announcement to confirm message delivery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1">
+      <c r="A46" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t>internal_messaging</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr">
         <is>
           <t>Internal Messaging</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>chat-dots</t>
         </is>
       </c>
-      <c r="E45" s="12" t="inlineStr">
+      <c r="E46" s="12" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
-        <is>
-          <t>roadmap</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="n">
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>roadmap</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr">
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
         <is>
           <t>messaging</t>
         </is>
       </c>
-      <c r="J45" s="3" t="inlineStr">
+      <c r="J46" s="3" t="inlineStr">
         <is>
           <t>Work chat scoped to your property. Department channels, direct messages, and file sharing — keeping work communication off WhatsApp and in a compliant, searchable system.</t>
         </is>

</xml_diff>